<commit_message>
chore(data): regenerate graph artifacts and processed dataset
Rebuild the processed dataset, features and edge arrays from the revised
pipeline, so the released graph carries the 2,000 km distance cap the
experiments apply.
</commit_message>
<xml_diff>
--- a/data/has_dash_records.xlsx
+++ b/data/has_dash_records.xlsx
@@ -1018,7 +1018,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>alkaline igneous rock</t>
+          <t>igneous rock</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1464,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>alkaline igneous rock</t>
+          <t>igneous rock (inferred, low confidence)</t>
         </is>
       </c>
     </row>
@@ -1494,7 +1494,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>alkaline igneous / carbonatite (inferred, medium confidence)</t>
+          <t>felsic igneous or sedimentary rock (inferred, low confidence)</t>
         </is>
       </c>
     </row>
@@ -2648,7 +2648,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>alkaline igneous / carbonatite (inferred, medium confidence)</t>
+          <t>igneous-related hydrothermal rock (inferred, low confidence)</t>
         </is>
       </c>
     </row>
@@ -3064,7 +3064,7 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>alkaline igneous rock</t>
+          <t>igneous rock</t>
         </is>
       </c>
     </row>
@@ -4080,7 +4080,7 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>alkaline igneous rock</t>
+          <t>igneous rock (inferred, low confidence)</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>alkaline igneous rock</t>
+          <t>igneous rock</t>
         </is>
       </c>
     </row>
@@ -4488,7 +4488,7 @@
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>alkaline igneous rock</t>
+          <t>igneous rock</t>
         </is>
       </c>
     </row>
@@ -4784,7 +4784,7 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>alkaline igneous rock</t>
+          <t>igneous rock (inferred, low confidence)</t>
         </is>
       </c>
     </row>
@@ -4814,7 +4814,7 @@
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>alkaline igneous rock</t>
+          <t>igneous rock (inferred, low confidence)</t>
         </is>
       </c>
     </row>
@@ -4904,7 +4904,7 @@
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>alkaline igneous rock</t>
+          <t>igneous rock</t>
         </is>
       </c>
     </row>
@@ -4934,7 +4934,7 @@
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>alkaline igneous rock</t>
+          <t>igneous rock</t>
         </is>
       </c>
     </row>
@@ -5234,7 +5234,7 @@
       </c>
       <c r="F162" t="inlineStr">
         <is>
-          <t>alkaline igneous rock</t>
+          <t>igneous rock (inferred, low confidence)</t>
         </is>
       </c>
     </row>

</xml_diff>